<commit_message>
Some folder structure modification
</commit_message>
<xml_diff>
--- a/Day-12-VLOOKUP/Day-12-VLOOKUP.xlsx
+++ b/Day-12-VLOOKUP/Day-12-VLOOKUP.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\90_Day_Data_Analytics\Day-12-VLOOKUP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{AA8875FB-00AF-4311-BCA7-34124CA29BA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43B7DA91-DE5F-4FC0-AEEE-296C0399655B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11280" xr2:uid="{9593C40E-69F7-409E-A99B-1F296548BDC0}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="9">
   <si>
     <t>Order_ID</t>
   </si>
@@ -59,6 +59,9 @@
   </si>
   <si>
     <t>FetchPrice</t>
+  </si>
+  <si>
+    <t>TV</t>
   </si>
 </sst>
 </file>
@@ -129,7 +132,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -142,6 +145,9 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -456,7 +462,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8AAD0D00-4C92-4B47-8339-D3DF188B238A}">
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:C10"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="10.28515625" customWidth="1"/>
@@ -531,6 +537,15 @@
       <c r="B9" s="4">
         <f>VLOOKUP(A9,Sheet2!A:B,2,0)</f>
         <v>3000</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="B10" s="4" t="e">
+        <f>VLOOKUP(A10,Sheet2!A:B,2,0)</f>
+        <v>#N/A</v>
       </c>
     </row>
   </sheetData>

</xml_diff>